<commit_message>
paper run 2026-10-28 10:36
</commit_message>
<xml_diff>
--- a/reports/2026-10-28.xlsx
+++ b/reports/2026-10-28.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -677,7 +677,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -687,75 +687,87 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>159.46</v>
+        <v>164.35</v>
       </c>
       <c r="E15" t="n">
-        <v>4.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>159.46</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="n">
-        <v>159.46</v>
-      </c>
-      <c r="E17" t="n">
-        <v>4.4</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>323.81</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" t="n">
-        <v>159.46</v>
-      </c>
-      <c r="E19" t="n">
-        <v>4.4</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>164.35</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -771,55 +783,62 @@
         <v>4.4</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>164.35</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>159.46</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4.4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" t="n">
-        <v>4.4</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>По окнам</t>
+          <t>По активам</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -841,7 +860,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -857,7 +876,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -879,7 +898,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -895,7 +914,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По часам</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -917,7 +936,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -933,7 +952,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>По силе движения</t>
+          <t>По цене входа</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -955,7 +974,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -971,7 +990,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>По направлению</t>
+          <t>По силе движения</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -993,16 +1012,54 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
         <v>4.4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
paper run 2026-10-28 17:54
</commit_message>
<xml_diff>
--- a/reports/2026-10-28.xlsx
+++ b/reports/2026-10-28.xlsx
@@ -681,13 +681,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>164.35</v>
+        <v>328.17</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -726,13 +726,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>323.81</v>
+        <v>487.63</v>
       </c>
       <c r="E18" t="n">
         <v>4.4</v>
@@ -752,13 +752,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>164.35</v>
+        <v>328.17</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -797,13 +797,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>164.35</v>
+        <v>328.17</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
paper run 2026-10-29 03:56
</commit_message>
<xml_diff>
--- a/reports/2026-10-28.xlsx
+++ b/reports/2026-10-28.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,49 @@
       </c>
       <c r="K2" t="n">
         <v>4.4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-28T23:11:16.335996+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F3" t="n">
+        <v>14.56</v>
+      </c>
+      <c r="G3" t="n">
+        <v>28</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.757</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.00106</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>13.44</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +593,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -560,7 +603,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -590,7 +633,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4.4</v>
+        <v>17.84</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +643,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4.4</v>
+        <v>17.84</v>
       </c>
     </row>
     <row r="8">
@@ -630,7 +673,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4245.809999999999</v>
+        <v>4263.149999999999</v>
       </c>
     </row>
     <row r="12">
@@ -681,16 +724,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>328.17</v>
+        <v>634.48</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>13.44</v>
       </c>
     </row>
     <row r="16">
@@ -722,88 +765,100 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>487.63</v>
+        <v>110.35</v>
       </c>
       <c r="E18" t="n">
-        <v>4.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" t="n">
+        <v>683.59</v>
+      </c>
+      <c r="E19" t="n">
+        <v>17.84</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>2</v>
-      </c>
-      <c r="C20" t="n">
-        <v>2</v>
-      </c>
-      <c r="D20" t="n">
-        <v>328.17</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>159.46</v>
+        <v>524.13</v>
       </c>
       <c r="E21" t="n">
-        <v>4.4</v>
+        <v>13.44</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>159.46</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4.4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>328.17</v>
+        <v>110.35</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -812,71 +867,78 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" t="n">
-        <v>159.46</v>
-      </c>
-      <c r="E24" t="n">
-        <v>4.4</v>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MAX_PER_WINDOW</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>110.35</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>328.17</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>355.42</v>
+      </c>
+      <c r="E27" t="n">
+        <v>17.84</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" t="n">
-        <v>4.4</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По окнам</t>
+          <t>По активам</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -898,23 +960,23 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>4.4</v>
+        <v>17.84</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -936,7 +998,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -946,111 +1008,121 @@
         <v>1</v>
       </c>
       <c r="D35" t="n">
+        <v>13.44</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
         <v>4.4</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="n">
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
         <v>4.4</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>13.44</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
-        <v>4.4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>13.44</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1061,6 +1133,98 @@
       </c>
       <c r="D44" t="n">
         <v>4.4</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>17.84</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>13.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>